<commit_message>
feat: included search and excel v2
</commit_message>
<xml_diff>
--- a/smt-backend/SMT_DATA/RESISTOR.xlsx
+++ b/smt-backend/SMT_DATA/RESISTOR.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="26">
   <si>
     <t>Reel ID</t>
   </si>
@@ -74,6 +74,21 @@
   </si>
   <si>
     <t>2026-08-13 12:00:00</t>
+  </si>
+  <si>
+    <t>REEL00012</t>
+  </si>
+  <si>
+    <t>PSRES99</t>
+  </si>
+  <si>
+    <t>LT-LIVE</t>
+  </si>
+  <si>
+    <t>OK</t>
+  </si>
+  <si>
+    <t>2026-08-20 07:35:38</t>
   </si>
 </sst>
 </file>
@@ -538,7 +553,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -638,8 +653,37 @@
         <v>20</v>
       </c>
     </row>
+    <row r="4" ht="22" customHeight="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" s="6">
+        <v>5000</v>
+      </c>
+      <c r="F4" s="6">
+        <v>5000</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>